<commit_message>
Record settled carton, packing, and ship-stats rules.
Flat pages stay outside the factory carton folder, WeChat zips use the short order code plus carton count, and the master table plus ship-stats workbook keep the confirmed 24-pack and store labels.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/1_Input_Raw/00_Master_Reference/2026.7.20桌布当前产品总表.xlsx
+++ b/1_Input_Raw/00_Master_Reference/2026.7.20桌布当前产品总表.xlsx
@@ -1672,13 +1672,13 @@
         </is>
       </c>
       <c r="T3" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="U3" s="4" t="n">
-        <v>15.64</v>
+        <v>17.06</v>
       </c>
       <c r="V3" s="4" t="n">
-        <v>17.02</v>
+        <v>18.44</v>
       </c>
       <c r="W3" s="16">
         <f>11.99*0.4*T3</f>
@@ -1752,13 +1752,13 @@
         </is>
       </c>
       <c r="T4" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>15.64</v>
+        <v>17.06</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>17.02</v>
+        <v>18.44</v>
       </c>
       <c r="W4" s="16">
         <f>14.99*0.4*T4</f>
@@ -1795,13 +1795,13 @@
         </is>
       </c>
       <c r="H5" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>15.64</v>
+        <v>17.06</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>17.02</v>
+        <v>18.44</v>
       </c>
       <c r="K5" s="16">
         <f>11.99*0.4*H5</f>
@@ -1834,13 +1834,13 @@
         </is>
       </c>
       <c r="T5" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="U5" s="4" t="n">
-        <v>15.64</v>
+        <v>17.06</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>17.02</v>
+        <v>18.44</v>
       </c>
       <c r="W5" s="16">
         <f>14.99*0.4*T5</f>
@@ -1875,13 +1875,13 @@
         </is>
       </c>
       <c r="H6" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>15.64</v>
+        <v>17.06</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>17.02</v>
+        <v>18.44</v>
       </c>
       <c r="K6" s="16">
         <f>14.99*0.4*H6</f>
@@ -1936,13 +1936,13 @@
         </is>
       </c>
       <c r="H7" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>15.64</v>
+        <v>17.06</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>17.02</v>
+        <v>18.44</v>
       </c>
       <c r="K7" s="16">
         <f>14.99*0.4*H7</f>
@@ -2018,13 +2018,13 @@
         </is>
       </c>
       <c r="H8" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>15.64</v>
+        <v>17.06</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>17.02</v>
+        <v>18.44</v>
       </c>
       <c r="K8" s="16">
         <f>14.99*0.4*H8</f>

</xml_diff>